<commit_message>
Banque de 20 thèmes pointus, annonce « T'es con ou connoisseur en… »
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4e3JGtiCx8jxBb2JR7Gh3
</commit_message>
<xml_diff>
--- a/themes.xlsx
+++ b/themes.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -484,12 +484,12 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Quel organe pompe le sang dans tout le corps ?</t>
+          <t>Contre quoi le Titanic s’est-il heurté ?</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Le cœur</t>
+          <t>Un iceberg</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -509,12 +509,12 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Combien de dents a un adulte, dents de sagesse comprises ?</t>
+          <t>Dans quel océan le Titanic a-t-il coulé ?</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>L’Atlantique (Nord)</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -534,12 +534,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus grand organe du corps humain ?</t>
+          <t>En quelle année le Titanic a-t-il coulé ?</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>La peau</t>
+          <t>1912</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -559,12 +559,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Quel est l’os le plus long du corps ?</t>
+          <t>Quel acteur joue Jack dans le film de 1997 ?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Le fémur</t>
+          <t>Leonardo DiCaprio</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -584,12 +584,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Où se trouve l’étrier, le plus petit os du corps ?</t>
+          <t>Vers quelle ville le Titanic faisait-il route ?</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Dans l’oreille (moyenne)</t>
+          <t>New York</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -609,12 +609,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Quel organe produit l’insuline ?</t>
+          <t>Qui a réalisé le film Titanic de 1997 ?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Le pancréas</t>
+          <t>James Cameron</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -634,12 +634,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Quel groupe sanguin est dit « donneur universel » ?</t>
+          <t>De quel port anglais le Titanic est-il parti ?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>O négatif</t>
+          <t>Southampton</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -659,12 +659,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Quelle protéine transporte l’oxygène dans le sang ?</t>
+          <t>Dans quel port français le Titanic a-t-il fait escale ?</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>L’hémoglobine</t>
+          <t>Cherbourg</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -684,12 +684,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Combien d’os compte environ le squelette d’un adulte ?</t>
+          <t>Quelle compagnie maritime exploitait le Titanic ?</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>La White Star Line</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Corps humain</t>
+          <t>Titanic</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -709,12 +709,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appellent les cellules principales du foie ?</t>
+          <t>Comment s’appelait le commandant du Titanic ?</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Les hépatocytes</t>
+          <t>Edward Smith</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -734,12 +734,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la formule chimique de l’eau ?</t>
+          <t>Dans quelle ville se trouve la tour Eiffel ?</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>H₂O</t>
+          <t>Paris</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -759,12 +759,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Quel gaz respirons-nous pour vivre ?</t>
+          <t>Quel ingénieur a donné son nom à la tour ?</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>L’oxygène</t>
+          <t>Gustave Eiffel</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -784,12 +784,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Quel est le symbole chimique de l’or ?</t>
+          <t>Pour quel événement la tour a-t-elle été construite ?</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Au</t>
+          <t>L’Exposition universelle de 1889</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -809,12 +809,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Quel gaz rend la voix aiguë quand on l’inhale ?</t>
+          <t>Combien d’étages de la tour sont ouverts au public ?</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>L’hélium</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -834,12 +834,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Quel est le symbole chimique du fer ?</t>
+          <t>En quel métal la tour est-elle construite ?</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>En fer</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -859,12 +859,12 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Quel élément porte le numéro atomique 1 ?</t>
+          <t>Quelle est sa hauteur, à 10 mètres près ?</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>L’hydrogène</t>
+          <t>Environ 330 m</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -884,12 +884,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Quel métal est liquide à température ambiante ?</t>
+          <t>Tous les combien d’années la tour est-elle repeinte ?</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Le mercure</t>
+          <t>Environ tous les 7 ans</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -909,12 +909,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Qui a publié le tableau périodique des éléments en 1869 ?</t>
+          <t>Quel gratte-ciel lui a ravi le titre de plus haute construction du monde en 1930 ?</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Dmitri Mendeleïev</t>
+          <t>Le Chrysler Building</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -934,12 +934,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Quel élément a pour symbole W ?</t>
+          <t>Quel escroc a « vendu » la tour Eiffel à un ferrailleur en 1925 ?</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Le tungstène</t>
+          <t>Victor Lustig</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Chimie</t>
+          <t>Tour Eiffel</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -959,12 +959,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Quel gaz noble radioactif peut s’accumuler dans les sous-sols ?</t>
+          <t>Quels ingénieurs de l’entreprise Eiffel ont dessiné les premiers plans de la tour ?</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Le radon</t>
+          <t>Maurice Koechlin et Émile Nouguier</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -984,12 +984,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>En quelle année a eu lieu la prise de la Bastille ?</t>
+          <t>Qui a été le premier homme à marcher sur la Lune ?</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>Neil Armstrong</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Quel roi est surnommé le Roi-Soleil ?</t>
+          <t>En quelle année l’homme a-t-il marché sur la Lune pour la première fois ?</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Louis XIV</t>
+          <t>1969</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Sur quelle île Napoléon est-il mort ?</t>
+          <t>Quel pays a envoyé les premiers hommes sur la Lune ?</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Sainte-Hélène</t>
+          <t>Les États-Unis</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Quelle héroïne a été brûlée à Rouen en 1431 ?</t>
+          <t>Qui a été le deuxième homme à marcher sur la Lune ?</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Jeanne d’Arc</t>
+          <t>Buzz Aldrin</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>En quelle année les Françaises ont-elles voté pour la première fois ?</t>
+          <t>Comment s’appelait la mission du premier alunissage ?</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>1945 (droit accordé en 1944)</t>
+          <t>Apollo 11</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -1109,12 +1109,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Quel roi a été guillotiné en janvier 1793 ?</t>
+          <t>Quel astronaute est resté en orbite pendant que les deux autres marchaient sur la Lune ?</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Louis XVI</t>
+          <t>Michael Collins</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -1134,12 +1134,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Quelle bataille François Ier a-t-il gagnée en 1515 ?</t>
+          <t>Quel nom portait le module lunaire d’Apollo 11 ?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Marignan</t>
+          <t>Eagle</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -1159,12 +1159,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Quel édit de 1598 accorde la liberté de culte aux protestants ?</t>
+          <t>Quelle fusée a lancé Apollo 11 ?</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>L’édit de Nantes</t>
+          <t>Saturn V</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Quel président de la République est tombé d’un train en pyjama en 1920 ?</t>
+          <t>Dans quelle zone de la Lune Apollo 11 s’est-il posé ?</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Paul Deschanel</t>
+          <t>La mer de la Tranquillité</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Histoire de France</t>
+          <t>Premiers pas sur la Lune</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Quel traité de 843 partage l’empire de Charlemagne entre ses petits-fils ?</t>
+          <t>Combien d’hommes au total ont marché sur la Lune ?</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Le traité de Verdun</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Combien de lettres compte l’alphabet français ?</t>
+          <t>Quel volcan a enseveli Pompéi ?</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>Le Vésuve</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la femelle du cheval ?</t>
+          <t>Dans quel pays se trouve Pompéi ?</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>La jument</t>
+          <t>L’Italie</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Quel est le pluriel de « œil » ?</t>
+          <t>Près de quelle grande ville se trouve Pompéi ?</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Yeux</t>
+          <t>Naples</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le petit signe sous le c de « ça » ?</t>
+          <t>En quelle année a eu lieu l’éruption qui a détruit Pompéi ?</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>La cédille</t>
+          <t>79 après J.-C.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -1334,12 +1334,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on un mot qui se lit dans les deux sens, comme « kayak » ?</t>
+          <t>Sous quoi la ville a-t-elle été ensevelie ?</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Un palindrome</t>
+          <t>Des cendres et des pierres ponces</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -1359,12 +1359,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Citez trois des sept noms en -ou qui prennent un x au pluriel.</t>
+          <t>Que signifie l’inscription « Cave canem » d’une célèbre mosaïque de Pompéi ?</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Bijou, caillou, chou, genou, hibou, joujou, pou</t>
+          <t>Attention au chien</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -1384,12 +1384,12 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on l’association de deux mots contradictoires, comme « obscure clarté » ?</t>
+          <t>Quelle ville voisine a été détruite par la même éruption ?</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Un oxymore</t>
+          <t>Herculanum</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Combien de lettres compte « anticonstitutionnellement » ?</t>
+          <t>Quel auteur latin a raconté l’éruption dans deux lettres à Tacite ?</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>Pline le Jeune</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -1434,12 +1434,12 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on une phrase qui contient toutes les lettres de l’alphabet ?</t>
+          <t>Quel savant romain est mort pendant l’éruption ?</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Un pangramme</t>
+          <t>Pline l’Ancien</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Langue française</t>
+          <t>Pompéi</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -1459,12 +1459,12 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le signe typographique « ¶ » ?</t>
+          <t>Quel archéologue a eu l’idée de couler du plâtre dans les vides laissés par les corps ?</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Le pied-de-mouche</t>
+          <t>Giuseppe Fiorelli</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Quel savant a formulé la gravitation après, dit-on, la chute d’une pomme ?</t>
+          <t>En quelle année le mur de Berlin est-il tombé ?</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Isaac Newton</t>
+          <t>1989</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -1509,12 +1509,12 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Quel physicien est célèbre pour la formule E = mc² ?</t>
+          <t>Quel pays le Mur coupait-il en deux ?</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
+          <t>L’Allemagne</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -1534,12 +1534,12 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Quels frères ont inventé le cinématographe ?</t>
+          <t>En quelle année le mur de Berlin a-t-il été construit ?</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Les frères Lumière</t>
+          <t>1961</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -1559,12 +1559,12 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Quel Français a mis au point le vaccin contre la rage ?</t>
+          <t>Quel sigle désignait l’Allemagne de l’Est ?</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Louis Pasteur</t>
+          <t>La RDA</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -1584,12 +1584,12 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’écriture en relief pour les personnes aveugles ?</t>
+          <t>Quel président américain a déclaré « Ich bin ein Berliner » en 1963 ?</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Le braille</t>
+          <t>John F. Kennedy</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Qui a inventé la machine à calculer appelée Pascaline ?</t>
+          <t>Quel était le point de passage le plus célèbre entre Berlin-Est et Berlin-Ouest ?</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Blaise Pascal</t>
+          <t>Checkpoint Charlie</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Qui a découvert la pénicilline en 1928 ?</t>
+          <t>Quel violoncelliste a joué au pied du Mur en novembre 1989 ?</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Alexander Fleming</t>
+          <t>Mstislav Rostropovitch</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Quelle scientifique a reçu deux prix Nobel dans deux sciences différentes ?</t>
+          <t>Comment s’appelait la police politique de la RDA ?</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Marie Curie</t>
+          <t>La Stasi</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -1684,12 +1684,12 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Quel Français a réalisé la plus ancienne photographie connue, vers 1827 ?</t>
+          <t>Quel porte-parole a annoncé par erreur l’ouverture immédiate des frontières le 9 novembre 1989 ?</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Nicéphore Niépce</t>
+          <t>Günter Schabowski</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Inventions et découvertes</t>
+          <t>Mur de Berlin</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -1709,12 +1709,12 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Quel ingénieur a breveté un moteur à explosion en 1860 ?</t>
+          <t>Quelle était la longueur totale du Mur autour de Berlin-Ouest, à 10 km près ?</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Étienne Lenoir</t>
+          <t>Environ 155 km</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -1734,12 +1734,12 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Quel outil sert à enfoncer un clou ?</t>
+          <t>De quel pays vient IKEA ?</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Le marteau</t>
+          <t>La Suède</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -1759,12 +1759,12 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Avec quoi vérifie-t-on qu’une étagère est bien droite ?</t>
+          <t>Quel plat emblématique sert le restaurant IKEA ?</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Un niveau à bulle</t>
+          <t>Les boulettes de viande</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -1784,12 +1784,12 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle une vis dont l’empreinte est en croix ?</t>
+          <t>Avec quel outil fourni monte-t-on la plupart des meubles IKEA ?</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Une vis cruciforme</t>
+          <t>Une clé Allen (clé hexagonale)</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -1809,12 +1809,12 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Que met-on dans un mur avant la vis pour qu’elle tienne ?</t>
+          <t>Comment s’appelle la bibliothèque la plus célèbre d’IKEA ?</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Une cheville</t>
+          <t>Billy</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -1834,12 +1834,12 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Quelle scie électrique permet de découper des courbes ?</t>
+          <t>À qui correspondent les lettres I et K de IKEA ?</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>La scie sauteuse</t>
+          <t>Ingvar Kamprad, le fondateur</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Quelle forme a une empreinte de vis Torx ?</t>
+          <t>Comment s’appelle le fauteuil IKEA en bois courbé vendu depuis les années 1970 ?</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Une étoile à six branches</t>
+          <t>Poäng</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
@@ -1884,12 +1884,12 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’outil manuel pour couper du carrelage ?</t>
+          <t>Comment s’appelle la peluche requin bleue d’IKEA ?</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>La carrelette (coupe-carreau)</t>
+          <t>Blåhaj</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
@@ -1909,12 +1909,12 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Quelle colle bicomposant mélange une résine et un durcisseur ?</t>
+          <t>En quelle année IKEA a-t-il été fondé ?</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>La colle époxy</t>
+          <t>1943</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -1934,12 +1934,12 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Quel appareil mesure à la fois tension, intensité et résistance ?</t>
+          <t>Dans quelle ville a ouvert le premier magasin IKEA en France ?</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Le multimètre</t>
+          <t>Bobigny</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Bricolage</t>
+          <t>IKEA</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’évasement conique qui permet de noyer une tête de vis ?</t>
+          <t>À quoi correspondent les lettres E et A de IKEA ?</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Une fraisure</t>
+          <t>Elmtaryd et Agunnaryd, la ferme et le village du fondateur</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Quel est l’ingrédient principal d’une omelette ?</t>
+          <t>Avec quel féculent mange-t-on traditionnellement la raclette ?</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Les œufs</t>
+          <t>Les pommes de terre</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Quelle sauce froide se fait avec un jaune d’œuf et de l’huile ?</t>
+          <t>De quel pays la raclette est-elle originaire ?</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>La mayonnaise</t>
+          <t>La Suisse</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -2034,12 +2034,12 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Combien de minutes environ cuit un œuf à la coque ?</t>
+          <t>Quels petits légumes au vinaigre accompagnent la raclette ?</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>3 minutes</t>
+          <t>Les cornichons (et petits oignons)</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Quels sont les trois ingrédients de base de la béchamel ?</t>
+          <t>Comment appelle-t-on les petites poêles de l’appareil à raclette ?</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Beurre, farine, lait</t>
+          <t>Les coupelles (ou poêlons)</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le bouquet de thym, laurier et persil ficelé ensemble ?</t>
+          <t>D’où vient le nom « raclette » ?</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Le bouquet garni</t>
+          <t>On racle le fromage fondu de la demi-meule</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -2109,12 +2109,12 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la découpe en fins bâtonnets ?</t>
+          <t>Quelle viande séchée suisse accompagne souvent la raclette ?</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>La julienne</t>
+          <t>La viande des Grisons</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -2134,12 +2134,12 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Quelle sauce chaude au beurre et aux jaunes d’œufs se parfume à l’estragon ?</t>
+          <t>De quel canton suisse vient la Raclette AOP ?</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>La béarnaise</t>
+          <t>Le Valais</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le mélange de beurre et de farine cuits qui sert à lier une sauce ?</t>
+          <t>La Raclette du Valais AOP est-elle faite au lait cru ou pasteurisé ?</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Un roux</t>
+          <t>Au lait cru</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -2184,12 +2184,12 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la garniture de carotte, oignon et céleri coupés en dés ?</t>
+          <t>Quel vin blanc valaisan accompagne traditionnellement la raclette ?</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>La mirepoix</t>
+          <t>Le fendant</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Cuisine</t>
+          <t>Raclette</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -2209,12 +2209,12 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Quelle réaction chimique fait dorer la viande à la cuisson ?</t>
+          <t>De quel cépage est fait le fendant ?</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>La réaction de Maillard</t>
+          <t>Le chasselas</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -2234,12 +2234,12 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la monnaie utilisée en France ?</t>
+          <t>Comment s’appelle le café court et serré qu’on boit au comptoir ?</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>L’euro</t>
+          <t>L’expresso</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Comment dit-on quand son compte bancaire est dans le négatif ?</t>
+          <t>Quel café italien est surmonté de lait moussé ?</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Être à découvert</t>
+          <t>Le cappuccino</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -2284,12 +2284,12 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Que signifie RIB ?</t>
+          <t>Quelle molécule stimulante contient le café ?</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Relevé d’identité bancaire</t>
+          <t>La caféine</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -2309,12 +2309,12 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>En quelle année les pièces et billets en euros sont-ils arrivés dans les poches ?</t>
+          <t>Quel café italien est un expresso « taché » d’un peu de mousse de lait ?</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>Le macchiato</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
@@ -2334,12 +2334,12 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Combien de francs valait un euro, arrondi au centime ?</t>
+          <t>Quelles sont les deux principales espèces de caféier cultivées ?</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>6,56 francs</t>
+          <t>L’arabica et le robusta</t>
         </is>
       </c>
     </row>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
@@ -2359,12 +2359,12 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Quelle institution fixe les taux directeurs de la zone euro ?</t>
+          <t>Quel pays est le premier producteur de café au monde ?</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>La Banque centrale européenne (BCE)</t>
+          <t>Le Brésil</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -2384,12 +2384,12 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus gros billet en euros encore émis ?</t>
+          <t>Entre arabica et robusta, lequel contient le plus de caféine ?</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Le billet de 200 €</t>
+          <t>Le robusta</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -2409,12 +2409,12 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Quel sigle désigne le taux qui inclut tous les frais d’un crédit ?</t>
+          <t>De quel pays le caféier est-il originaire ?</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Le TAEG</t>
+          <t>L’Éthiopie</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -2434,12 +2434,12 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Que signifie CAC dans CAC 40 ?</t>
+          <t>Selon la légende, quel berger a découvert le café grâce à ses chèvres excitées ?</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Cotation assistée en continu</t>
+          <t>Kaldi</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Argent et banque</t>
+          <t>Café</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -2459,12 +2459,12 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelait l’unité de compte européenne qui a précédé l’euro ?</t>
+          <t>Quel café indonésien est fait de grains digérés par une civette ?</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>L’ECU</t>
+          <t>Le kopi luwak</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -2484,12 +2484,12 @@
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Que doit faire un conducteur face à un feu rouge ?</t>
+          <t>Comment appelle-t-on ouvrir une bouteille d’un coup de sabre ?</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>S’arrêter</t>
+          <t>Sabrer</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la vitesse maximale sur autoroute par temps sec ?</t>
+          <t>Quel moine est associé à la légende de l’invention du champagne ?</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>130 km/h</t>
+          <t>Dom Pérignon</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -2534,12 +2534,12 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Quelle forme a un panneau stop ?</t>
+          <t>Quelle ville est la capitale historique du champagne, avec sa cathédrale des sacres ?</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Octogonale</t>
+          <t>Reims</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -2559,12 +2559,12 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la vitesse maximale par défaut en agglomération ?</t>
+          <t>Comment s’appelle l’armature en fil de fer qui retient le bouchon ?</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>50 km/h</t>
+          <t>Le muselet</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>De quelle couleur sont les panneaux de travaux temporaires ?</t>
+          <t>Que veut dire « brut » sur une bouteille de champagne ?</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Jaunes</t>
+          <t>Qu’il est peu sucré</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -2609,12 +2609,12 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Combien de points compte un permis de conduire complet ?</t>
+          <t>Quels sont les trois principaux cépages du champagne ?</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>Chardonnay, pinot noir, pinot meunier</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -2634,12 +2634,12 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Quel est le taux d’alcool maximal pour un conducteur confirmé, en grammes par litre de sang ?</t>
+          <t>Que signifie « blanc de blancs » ?</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>0,5 g/L</t>
+          <t>Fait uniquement de raisins blancs</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -2659,12 +2659,12 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la vitesse maximale sur autoroute par temps de pluie ?</t>
+          <t>Combien de litres contient un jéroboam de champagne ?</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>110 km/h</t>
+          <t>3 litres</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -2684,12 +2684,12 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Avec combien de points démarre un permis probatoire ?</t>
+          <t>Comment s’appelle l’opération qui expulse le dépôt de levures du col de la bouteille ?</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>6 points</t>
+          <t>Le dégorgement</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Code de la route</t>
+          <t>Champagne</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -2709,12 +2709,12 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Quel est le taux d’alcool maximal pour un jeune conducteur, en grammes par litre de sang ?</t>
+          <t>Comment appelle-t-on un collectionneur de capsules de champagne ?</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>0,2 g/L</t>
+          <t>Un placomusophile</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -2734,12 +2734,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Combien de mois dure environ une grossesse ?</t>
+          <t>Quelle marque fabriquait la 2CV ?</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>9 mois</t>
+          <t>Citroën</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -2759,12 +2759,12 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on le lait en poudre pour nourrissons ?</t>
+          <t>Que signifie « CV » dans 2CV ?</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Le lait infantile</t>
+          <t>Chevaux (fiscaux)</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2776,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
@@ -2784,12 +2784,12 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Vers quel âge un bébé fait-il généralement ses premiers pas ?</t>
+          <t>Quel surnom affectueux donne-t-on à la 2CV ?</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Vers 1 an</t>
+          <t>La deudeuche (ou deuche)</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
@@ -2809,12 +2809,12 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Combien de dents de lait a un enfant ?</t>
+          <t>En quoi est le toit d’origine de la 2CV ?</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>En toile</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la zone molle sur le crâne du nourrisson ?</t>
+          <t>En quelle année la 2CV a-t-elle été présentée au Salon de Paris ?</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>La fontanelle</t>
+          <t>1948</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2851,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -2859,12 +2859,12 @@
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Contre quelles maladies protège le vaccin ROR ?</t>
+          <t>Selon le cahier des charges, que devait-elle transporter à travers un champ sans le casser ?</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Rougeole, oreillons, rubéole</t>
+          <t>Un panier d’œufs</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le premier lait, très riche, produit après l’accouchement ?</t>
+          <t>En quelle année la production de la 2CV s’est-elle arrêtée ?</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Le colostrum</t>
+          <t>1990</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la toute première selle du nouveau-né ?</t>
+          <t>Dans quel pays la dernière 2CV a-t-elle été fabriquée ?</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Le méconium</t>
+          <t>Le Portugal</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
@@ -2934,12 +2934,12 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Quel score évalue l’état du nouveau-né juste après la naissance ?</t>
+          <t>Quelle version de la 2CV avait deux moteurs, un à l’avant et un à l’arrière ?</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Le score d’Apgar</t>
+          <t>La 2CV Sahara</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Bébés et parents</t>
+          <t>2CV</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le réflexe du nourrisson qui écarte les bras quand il sursaute ?</t>
+          <t>Quel patron de Citroën a lancé le projet de la 2CV ?</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Le réflexe de Moro</t>
+          <t>Pierre-Jules Boulanger</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
@@ -2984,12 +2984,12 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Quel film de 2001 suit une jeune serveuse de Montmartre ?</t>
+          <t>Dans quelle école de sorcellerie étudie Harry ?</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Le Fabuleux Destin d’Amélie Poulain</t>
+          <t>Poudlard</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
@@ -3009,12 +3009,12 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la récompense suprême du Festival de Cannes ?</t>
+          <t>Qui a écrit la saga Harry Potter ?</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>La Palme d’or</t>
+          <t>J. K. Rowling</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
@@ -3034,12 +3034,12 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la récompense du cinéma français remise chaque année ?</t>
+          <t>Quelle forme a la cicatrice de Harry ?</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Le César</t>
+          <t>Un éclair</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
@@ -3059,12 +3059,12 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Quel film de Dany Boon se déroule à Bergues ?</t>
+          <t>Comment s’appellent les deux meilleurs amis de Harry ?</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Bienvenue chez les Ch’tis</t>
+          <t>Ron et Hermione</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
@@ -3084,12 +3084,12 @@
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>Quel film de 2011 réunit Omar Sy et François Cluzet ?</t>
+          <t>Dans quelle maison est Harry ?</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>Intouchables</t>
+          <t>Gryffondor</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
@@ -3109,12 +3109,12 @@
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>Quel réalisateur a signé « Le Grand Bleu » et « Léon » ?</t>
+          <t>De quel quai part le Poudlard Express ?</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Luc Besson</t>
+          <t>Le quai 9 ¾</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
@@ -3134,12 +3134,12 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>Qui a réalisé « Les Quatre Cents Coups » en 1959 ?</t>
+          <t>Comment s’appelle la chouette de Harry ?</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>François Truffaut</t>
+          <t>Hedwige</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>Quel film français a remporté l’Oscar du meilleur film en 2012 ?</t>
+          <t>Quel est le vrai nom de Voldemort dans la version française ?</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>The Artist</t>
+          <t>Tom Elvis Jedusor</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
@@ -3184,12 +3184,12 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>Quel film de Jacques Demy, sorti en 1964, est entièrement chanté ?</t>
+          <t>Quelle forme prend le Patronus de Harry ?</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>Les Parapluies de Cherbourg</t>
+          <t>Un cerf</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Cinéma français</t>
+          <t>Harry Potter</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
@@ -3209,12 +3209,12 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>Qui a réalisé « Playtime » en 1967 ?</t>
+          <t>Quel est le deuxième prénom de Harry ?</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Jacques Tati</t>
+          <t>James</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
@@ -3234,12 +3234,12 @@
       </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
-          <t>Quelle chanteuse est associée à « La Vie en rose » ?</t>
+          <t>Qui est le père de Luke Skywalker ?</t>
         </is>
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>Édith Piaf</t>
+          <t>Dark Vador</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
@@ -3259,12 +3259,12 @@
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>Quel duo français casqué a sorti « Get Lucky » ?</t>
+          <t>Comment s’appelle le petit maître Jedi vert qui parle à l’envers ?</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>Daft Punk</t>
+          <t>Yoda</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
@@ -3284,12 +3284,12 @@
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>Qui chante « Ne me quitte pas » ?</t>
+          <t>Comment s’appelle le copilote wookiee du Faucon Millenium ?</t>
         </is>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>Jacques Brel</t>
+          <t>Chewbacca</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
@@ -3309,12 +3309,12 @@
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>Quel groupe a sorti « L’Aventurier » ?</t>
+          <t>Comment s’appelle le petit droïde bleu et blanc ?</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>Indochine</t>
+          <t>R2-D2</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
@@ -3334,12 +3334,12 @@
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>Quel chanteur a créé « La Bohème » ?</t>
+          <t>Qui est le pilote du Faucon Millenium ?</t>
         </is>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>Charles Aznavour</t>
+          <t>Han Solo</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
@@ -3359,12 +3359,12 @@
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>Qui a écrit « Le Poinçonneur des Lilas » ?</t>
+          <t>Qui a créé Star Wars ?</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>Serge Gainsbourg</t>
+          <t>George Lucas</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
@@ -3384,12 +3384,12 @@
       </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
-          <t>Quel était le vrai nom de famille de Johnny Hallyday ?</t>
+          <t>Quel est le prénom de Dark Vador avant qu’il bascule du côté obscur ?</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>Smet</t>
+          <t>Anakin</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
@@ -3409,12 +3409,12 @@
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>Qui a représenté la France à l’Eurovision 2021 avec « Voilà » ?</t>
+          <t>En quelle année est sorti le premier film Star Wars ?</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>Barbara Pravi</t>
+          <t>1977</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
@@ -3434,12 +3434,12 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>Quel était le vrai prénom de Serge Gainsbourg ?</t>
+          <t>Sur quelle planète glacée s’ouvre « L’Empire contre-attaque » ?</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>Lucien</t>
+          <t>Hoth</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Chanson</t>
+          <t>Star Wars</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
@@ -3459,12 +3459,12 @@
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>Quelle chanson a donné à la France sa dernière victoire à l’Eurovision, en 1977 ?</t>
+          <t>Quel matricule portait Finn quand il était stormtrooper ?</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>« L’oiseau et l’enfant » (Marie Myriam)</t>
+          <t>FN-2187</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
@@ -3484,12 +3484,12 @@
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>Combien de joueurs par équipe sont sur un terrain de football ?</t>
+          <t>Comment s’appelle le père de la famille Simpson ?</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>Homer</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
@@ -3509,12 +3509,12 @@
       </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
-          <t>Tous les combien d’années ont lieu les Jeux olympiques d’été ?</t>
+          <t>Dans quelle ville vivent les Simpson ?</t>
         </is>
       </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
-          <t>Tous les 4 ans</t>
+          <t>Springfield</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
@@ -3534,12 +3534,12 @@
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>De quelle couleur est le maillot du leader du Tour de France ?</t>
+          <t>Où travaille Homer ?</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>Jaune</t>
+          <t>À la centrale nucléaire</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
@@ -3559,12 +3559,12 @@
       </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
-          <t>Quel tournoi du Grand Chelem se joue sur terre battue ?</t>
+          <t>Quelle bière boit Homer ?</t>
         </is>
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
-          <t>Roland-Garros</t>
+          <t>La Duff</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
@@ -3584,12 +3584,12 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>En quelle année la France a-t-elle gagné sa première Coupe du monde de football ?</t>
+          <t>De quel instrument joue Lisa ?</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>Du saxophone</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
@@ -3609,12 +3609,12 @@
       </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
-          <t>Combien de points vaut un essai au rugby ?</t>
+          <t>Comment s’appelle le patron d’Homer ?</t>
         </is>
       </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>Monsieur Burns</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Quelle distance mesure un marathon ?</t>
+          <t>Comment s’appelle le clown préféré de Bart ?</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>42,195 km</t>
+          <t>Krusty</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
@@ -3659,12 +3659,12 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Dans quelle ville ont eu lieu les premiers Jeux olympiques modernes, en 1896 ?</t>
+          <t>Qui a créé Les Simpson ?</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>Athènes</t>
+          <t>Matt Groening</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3676,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Quel Français a gagné le Tour de France cinq fois, la dernière en 1985 ?</t>
+          <t>Comment s’appelle le chien des Simpson en version française ?</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>Bernard Hinault</t>
+          <t>Petit Papa Noël</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Les Simpson</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
@@ -3709,12 +3709,12 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>Quelle est la longueur d’un court de tennis ?</t>
+          <t>Quel est le nom de famille d’Apu ?</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>23,77 m</t>
+          <t>Nahasapeemapetilon</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
@@ -3734,12 +3734,12 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>Quelle série suit six amis qui se retrouvent au Central Perk ?</t>
+          <t>De quelle ville anglaise viennent les Beatles ?</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>Friends</t>
+          <t>Liverpool</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
@@ -3759,12 +3759,12 @@
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Quelle série espagnole met en scène des braqueurs aux masques de Dalí ?</t>
+          <t>De quelle couleur est le sous-marin de leur célèbre chanson ?</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>La casa de papel</t>
+          <t>Jaune</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
@@ -3784,12 +3784,12 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Quelle série raconte la lutte pour le Trône de fer ?</t>
+          <t>Quel album montre les quatre Beatles sur un passage piéton ?</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>Game of Thrones</t>
+          <t>Abbey Road</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Quel est le métier de Walter White au début de « Breaking Bad » ?</t>
+          <t>Qui est le batteur des Beatles ?</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>Professeur de chimie</t>
+          <t>Ringo Starr</t>
         </is>
       </c>
     </row>
@@ -3826,7 +3826,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
@@ -3834,12 +3834,12 @@
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Dans quelle série Omar Sy s’inspire-t-il d’Arsène Lupin ?</t>
+          <t>Citez les quatre Beatles.</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>Lupin</t>
+          <t>John Lennon, Paul McCartney, George Harrison, Ringo Starr</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
@@ -3859,12 +3859,12 @@
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>Qui a créé « Kaamelott » ?</t>
+          <t>En quelle année les Beatles se sont-ils séparés ?</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>Alexandre Astier</t>
+          <t>1970</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
@@ -3884,12 +3884,12 @@
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>Dans quelle ville se déroule « Breaking Bad » ?</t>
+          <t>Dans quel club de Liverpool les Beatles ont-ils fait leurs débuts ?</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>Albuquerque</t>
+          <t>Le Cavern Club</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
@@ -3909,12 +3909,12 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la petite ville de « Stranger Things » ?</t>
+          <t>Dans quelle ville allemande les Beatles ont-ils joué avant de percer ?</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>Hawkins</t>
+          <t>Hambourg</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
@@ -3934,12 +3934,12 @@
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>Quelle entreprise de papier sert de décor à « The Office » américain ?</t>
+          <t>Comment s’appelait le manager des Beatles ?</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Dunder Mifflin</t>
+          <t>Brian Epstein</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Séries</t>
+          <t>Les Beatles</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
@@ -3959,12 +3959,12 @@
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>Quelle chaîne a diffusé « Les Soprano » ?</t>
+          <t>Quel est le vrai nom de Ringo Starr ?</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>HBO</t>
+          <t>Richard Starkey</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
@@ -3984,12 +3984,12 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Quel petit Gaulois a pour meilleur ami un livreur de menhirs ?</t>
+          <t>De quelle couleur est le maillot du leader du Tour ?</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Astérix</t>
+          <t>Jaune</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
@@ -4009,12 +4009,12 @@
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>Quel reporter a un chien nommé Milou ?</t>
+          <t>Sur quelle avenue le Tour se termine-t-il traditionnellement ?</t>
         </is>
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>Tintin</t>
+          <t>Les Champs-Élysées</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
@@ -4034,12 +4034,12 @@
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Qui a créé Tintin ?</t>
+          <t>Quel maillot porte le meilleur grimpeur ?</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>Hergé</t>
+          <t>Le maillot à pois (blanc à pois rouges)</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
@@ -4059,12 +4059,12 @@
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le capitaine ami de Tintin ?</t>
+          <t>De quelle couleur est le maillot du classement par points ?</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>Haddock</t>
+          <t>Vert</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
@@ -4084,12 +4084,12 @@
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le chef du village d’Astérix ?</t>
+          <t>À quel coureur américain a-t-on retiré sept victoires pour dopage ?</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>Abraracourcix</t>
+          <t>Lance Armstrong</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
@@ -4109,12 +4109,12 @@
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>Dans quelle ville a lieu le grand festival de la BD chaque mois de janvier ?</t>
+          <t>Quelle montée des Alpes est célèbre pour ses 21 virages ?</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
         <is>
-          <t>Angoulême</t>
+          <t>L’Alpe d’Huez</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
@@ -4134,12 +4134,12 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Qui a dessiné Astérix ?</t>
+          <t>Quel coureur belge surnommé « le Cannibale » a gagné cinq Tours ?</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>Albert Uderzo</t>
+          <t>Eddy Merckx</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
@@ -4159,12 +4159,12 @@
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>Quel est le vrai nom d’Hergé ?</t>
+          <t>En quelle année a eu lieu le premier Tour de France ?</t>
         </is>
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>Georges Remi</t>
+          <t>1903</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C150" s="2" t="n">
@@ -4184,12 +4184,12 @@
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Qui a créé Lucky Luke ?</t>
+          <t>Quel journal a créé le Tour de France ?</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>Morris</t>
+          <t>L’Auto</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Bande dessinée</t>
+          <t>Tour de France</t>
         </is>
       </c>
       <c r="C151" s="2" t="n">
@@ -4209,12 +4209,12 @@
       </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
-          <t>Quel auteur a créé « Blake et Mortimer » ?</t>
+          <t>Qui a remporté le premier Tour de France ?</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
-          <t>Edgar P. Jacobs</t>
+          <t>Maurice Garin</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
@@ -4234,12 +4234,12 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Quel animal a un très long cou et mange les feuilles en hauteur ?</t>
+          <t>Combien de couleurs y a-t-il sur un Rubik’s Cube classique ?</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>La girafe</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C153" s="2" t="n">
@@ -4259,12 +4259,12 @@
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>Quel reptile change de couleur et bouge ses yeux indépendamment ?</t>
+          <t>Combien de cases colorées compte chaque face du cube classique ?</t>
         </is>
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
-          <t>Le caméléon</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C154" s="2" t="n">
@@ -4284,12 +4284,12 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Quel est le seul mammifère capable de vraiment voler ?</t>
+          <t>Qui a inventé le Rubik’s Cube ?</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>La chauve-souris</t>
+          <t>Ernő Rubik</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C155" s="2" t="n">
@@ -4309,12 +4309,12 @@
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>Combien de cœurs a une pieuvre ?</t>
+          <t>De quel pays vient son inventeur ?</t>
         </is>
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>La Hongrie</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C156" s="2" t="n">
@@ -4334,12 +4334,12 @@
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Quel mammifère pond des œufs et a un bec de canard ?</t>
+          <t>Comment s’appelle la discipline qui consiste à résoudre le cube le plus vite possible ?</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>L’ornithorynque</t>
+          <t>Le speedcubing</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C157" s="2" t="n">
@@ -4359,12 +4359,12 @@
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>Combien de compartiments compte l’estomac d’une vache ?</t>
+          <t>En quelle année le Rubik’s Cube a-t-il été inventé ?</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1974</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C158" s="2" t="n">
@@ -4384,12 +4384,12 @@
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Quel oiseau est capable de voler en marche arrière ?</t>
+          <t>Sur un cube standard, quelle couleur est opposée au blanc ?</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>Le colibri</t>
+          <t>Le jaune</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C159" s="2" t="n">
@@ -4409,12 +4409,12 @@
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>Quel animal microscopique peut survivre dans le vide spatial ?</t>
+          <t>Comment appelle-t-on le nombre minimal de mouvements qui suffit à résoudre n’importe quelle position ?</t>
         </is>
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>Le tardigrade</t>
+          <t>Le nombre de Dieu</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C160" s="2" t="n">
@@ -4434,12 +4434,12 @@
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Quel poisson rendu célèbre par un film d’animation peut changer de sexe ?</t>
+          <t>Combien vaut ce nombre (en demi-tours comptés comme un mouvement) ?</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>Le poisson-clown</t>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Animaux bizarres</t>
+          <t>Rubik’s Cube</t>
         </is>
       </c>
       <c r="C161" s="2" t="n">
@@ -4459,12 +4459,12 @@
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>Quelle méduse est surnommée « l’immortelle » ?</t>
+          <t>Combien de combinaisons possibles compte le cube, en ordre de grandeur ?</t>
         </is>
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>Turritopsis dohrnii</t>
+          <t>Environ 43 milliards de milliards</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C162" s="2" t="n">
@@ -4484,12 +4484,12 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus grand océan du monde ?</t>
+          <t>De quel pays vient Lego ?</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>Le Pacifique</t>
+          <t>Le Danemark</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C163" s="2" t="n">
@@ -4509,12 +4509,12 @@
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus haut sommet du monde ?</t>
+          <t>Comment s’appellent les parcs d’attractions de la marque ?</t>
         </is>
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
-          <t>L’Everest</t>
+          <t>Legoland</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C164" s="2" t="n">
@@ -4534,12 +4534,12 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus grand pays du monde par sa superficie ?</t>
+          <t>En quelle matière sont fabriquées les briques Lego ?</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>La Russie</t>
+          <t>En plastique (ABS)</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C165" s="2" t="n">
@@ -4559,12 +4559,12 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus grand désert chaud du monde ?</t>
+          <t>Comment s’appelle le petit personnage Lego ?</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>Le Sahara</t>
+          <t>La minifigurine</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C166" s="2" t="n">
@@ -4584,12 +4584,12 @@
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus grand animal ayant jamais existé ?</t>
+          <t>Que signifie l’expression danoise « leg godt », à l’origine du nom ?</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>La baleine bleue</t>
+          <t>« Joue bien »</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C167" s="2" t="n">
@@ -4609,12 +4609,12 @@
       </c>
       <c r="D167" s="3" t="inlineStr">
         <is>
-          <t>Quel est le plus petit État du monde ?</t>
+          <t>En quelle matière Lego fabriquait-il ses premiers jouets ?</t>
         </is>
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
-          <t>Le Vatican</t>
+          <t>En bois</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C168" s="2" t="n">
@@ -4634,12 +4634,12 @@
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Quel pays est le plus peuplé du monde depuis 2023 ?</t>
+          <t>En quelle année la brique Lego moderne a-t-elle été brevetée ?</t>
         </is>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>L’Inde</t>
+          <t>1958</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C169" s="2" t="n">
@@ -4659,12 +4659,12 @@
       </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
-          <t>Quel fleuve est le plus souvent cité comme le plus long du monde ?</t>
+          <t>Qui a fondé Lego ?</t>
         </is>
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
-          <t>Le Nil (disputé avec l’Amazone)</t>
+          <t>Ole Kirk Christiansen</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C170" s="2" t="n">
@@ -4684,12 +4684,12 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>Quel est le lac le plus profond du monde ?</t>
+          <t>Dans quelle ville danoise se trouve le siège de Lego ?</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>Le lac Baïkal</t>
+          <t>Billund</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Records du monde</t>
+          <t>Lego</t>
         </is>
       </c>
       <c r="C171" s="2" t="n">
@@ -4709,12 +4709,12 @@
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>Quelle ville est le siège de gouvernement le plus haut du monde ?</t>
+          <t>De combien de façons peut-on assembler six briques 2×4 de même couleur, à 100 millions près ?</t>
         </is>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>La Paz (Bolivie)</t>
+          <t>915 103 765, environ 900 millions</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C172" s="2" t="n">
@@ -4734,12 +4734,12 @@
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « poser un lapin » ?</t>
+          <t>Quel film de Spielberg a rendu les requins terrifiants ?</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>Ne pas venir à un rendez-vous</t>
+          <t>Les Dents de la mer</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C173" s="2" t="n">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « avoir le cafard » ?</t>
+          <t>Le requin est-il un poisson ou un mammifère ?</t>
         </is>
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>Avoir des idées noires, être déprimé</t>
+          <t>Un poisson</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C174" s="2" t="n">
@@ -4784,12 +4784,12 @@
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « coûter les yeux de la tête » ?</t>
+          <t>Quel requin a la tête en forme de T ?</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>Être très cher</t>
+          <t>Le requin-marteau</t>
         </is>
       </c>
     </row>
@@ -4801,7 +4801,7 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C175" s="2" t="n">
@@ -4809,12 +4809,12 @@
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « tomber dans les pommes » ?</t>
+          <t>Quel est le plus grand requin, et le plus grand poisson du monde ?</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>S’évanouir</t>
+          <t>Le requin-baleine</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C176" s="2" t="n">
@@ -4834,12 +4834,12 @@
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « avoir un poil dans la main » ?</t>
+          <t>De quoi est fait le squelette d’un requin ?</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>Être paresseux</t>
+          <t>De cartilage</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C177" s="2" t="n">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « se faire rouler dans la farine » ?</t>
+          <t>Que deviennent les dents d’un requin quand il les perd ?</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>Se faire tromper</t>
+          <t>Elles repoussent, toute sa vie</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C178" s="2" t="n">
@@ -4884,12 +4884,12 @@
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « prendre la poudre d’escampette » ?</t>
+          <t>Quel requin préhistorique géant a disparu il y a environ 3,6 millions d’années ?</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>S’enfuir</t>
+          <t>Le mégalodon</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C179" s="2" t="n">
@@ -4909,12 +4909,12 @@
       </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « faire chou blanc » ?</t>
+          <t>Quel requin est le vertébré connu qui vit le plus longtemps ?</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>Échouer, ne rien obtenir</t>
+          <t>Le requin du Groenland</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C180" s="2" t="n">
@@ -4934,12 +4934,12 @@
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Au sens d’origine, que veut dire « tirer les marrons du feu » ?</t>
+          <t>Comment s’appellent les minuscules « dents » qui recouvrent la peau du requin ?</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>Prendre des risques dont un autre profite</t>
+          <t>Les denticules</t>
         </is>
       </c>
     </row>
@@ -4951,7 +4951,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Expressions françaises</t>
+          <t>Requins</t>
         </is>
       </c>
       <c r="C181" s="2" t="n">
@@ -4959,12 +4959,12 @@
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>Que veut dire « payer en monnaie de singe » ?</t>
+          <t>Comment s’appellent les organes qui permettent au requin de sentir les champs électriques ?</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>Payer en grimaces ou en belles paroles, donc ne pas payer</t>
+          <t>Les ampoules de Lorenzini</t>
         </is>
       </c>
     </row>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C182" s="2" t="n">
@@ -4984,12 +4984,12 @@
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’ustensile pour égoutter les pâtes ?</t>
+          <t>Quel oiseau se perche sur l’épaule des pirates dans les histoires ?</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>La passoire</t>
+          <t>Le perroquet</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C183" s="2" t="n">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on l’extrémité d’une baguette de pain ?</t>
+          <t>Comment s’appelle le pirate ennemi de Peter Pan ?</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>Le quignon (ou croûton)</t>
+          <t>Le capitaine Crochet</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C184" s="2" t="n">
@@ -5034,12 +5034,12 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le dessous du pied ?</t>
+          <t>Dans quel roman de Stevenson apparaît Long John Silver ?</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>La plante du pied</t>
+          <t>L’Île au trésor</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C185" s="2" t="n">
@@ -5059,12 +5059,12 @@
       </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le trou d’une aiguille ?</t>
+          <t>Comment s’appelle le drapeau noir à tête de mort ?</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>Le chas</t>
+          <t>Le Jolly Roger</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C186" s="2" t="n">
@@ -5084,12 +5084,12 @@
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Comment appelle-t-on un petit papier repositionnable pour noter un rappel ?</t>
+          <t>Qu’est-ce qui distingue un corsaire d’un pirate ?</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>Un pense-bête (post-it)</t>
+          <t>Il agit avec une autorisation de son souverain (lettre de marque)</t>
         </is>
       </c>
     </row>
@@ -5101,7 +5101,7 @@
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C187" s="2" t="n">
@@ -5109,12 +5109,12 @@
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’embout plastique au bout d’un lacet ?</t>
+          <t>Comment appelait-on les aventuriers qui pillaient les navires espagnols aux Caraïbes au XVIIe siècle ?</t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>L’aiglet (ou ferret)</t>
+          <t>Les flibustiers</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C188" s="2" t="n">
@@ -5134,12 +5134,12 @@
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la bague de métal qui tient la gomme au bout d’un crayon ?</t>
+          <t>Quel célèbre corsaire était originaire de Saint-Malo ?</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>La virole</t>
+          <t>Robert Surcouf</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C189" s="2" t="n">
@@ -5159,12 +5159,12 @@
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle le petit sillon entre le nez et la lèvre supérieure ?</t>
+          <t>Quel était le vrai nom de Barbe-Noire ?</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>Le philtrum</t>
+          <t>Edward Teach</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C190" s="2" t="n">
@@ -5184,12 +5184,12 @@
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’espace entre les deux sourcils ?</t>
+          <t>Quelle femme pirate naviguait avec Mary Read ?</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>La glabelle</t>
+          <t>Anne Bonny</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Mots méconnus</t>
+          <t>Pirates</t>
         </is>
       </c>
       <c r="C191" s="2" t="n">
@@ -5209,12 +5209,12 @@
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle l’odeur de la terre après la pluie ?</t>
+          <t>Quelle île au large de Madagascar a servi de repaire aux pirates ?</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>Le pétrichor</t>
+          <t>L’île Sainte-Marie</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C192" s="2" t="n">
@@ -5234,12 +5234,12 @@
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>Quel animal porte malheur quand il croise votre route ?</t>
+          <t>Quels animaux tirent le traîneau du Père Noël ?</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>Le chat noir</t>
+          <t>Des rennes</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C193" s="2" t="n">
@@ -5259,12 +5259,12 @@
       </c>
       <c r="D193" s="3" t="inlineStr">
         <is>
-          <t>Combien de feuilles a un trèfle porte-bonheur ?</t>
+          <t>Par où le Père Noël entre-t-il dans les maisons ?</t>
         </is>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Par la cheminée</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C194" s="2" t="n">
@@ -5284,12 +5284,12 @@
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Combien d’années de malheur promet un miroir cassé ?</t>
+          <t>Comment s’appelle le renne au nez rouge ?</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>7 ans</t>
+          <t>Rudolph</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C195" s="2" t="n">
@@ -5309,12 +5309,12 @@
       </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
-          <t>Sous quoi ne faut-il jamais passer ?</t>
+          <t>De quel saint le Père Noël est-il inspiré ?</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>Une échelle</t>
+          <t>Saint Nicolas</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C196" s="2" t="n">
@@ -5334,12 +5334,12 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Après avoir renversé du sel, par-dessus quelle épaule en jette-t-on une pincée ?</t>
+          <t>Quelle marque de soda a popularisé son image en rouge et blanc dans ses publicités des années 1930 ?</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>L’épaule gauche</t>
+          <t>Coca-Cola</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C197" s="2" t="n">
@@ -5359,12 +5359,12 @@
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>Selon la tradition, à qui était réservé le pain posé à l’envers ?</t>
+          <t>Dans quelle région du monde la tradition place-t-elle son village ?</t>
         </is>
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
-          <t>Au bourreau</t>
+          <t>La Laponie (Finlande)</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C198" s="2" t="n">
@@ -5384,12 +5384,12 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Quelle couleur de costume est bannie sur une scène de théâtre ?</t>
+          <t>Combien de rennes compte l’attelage classique, sans Rudolph ?</t>
         </is>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>Le vert</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C199" s="2" t="n">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>Quel mot ne faut-il jamais prononcer dans un théâtre ?</t>
+          <t>Dans quelle ville française La Poste répond-elle aux lettres au Père Noël ?</t>
         </is>
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
-          <t>« Corde »</t>
+          <t>Libourne</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C200" s="2" t="n">
@@ -5434,12 +5434,12 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Dans quel pays le chiffre 4 est-il redouté parce qu’il se prononce comme « mort » ?</t>
+          <t>Quel illustrateur a dessiné le Père Noël des publicités Coca-Cola ?</t>
         </is>
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>La Chine (aussi au Japon et en Corée)</t>
+          <t>Haddon Sundblom</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>Superstitions</t>
+          <t>Père Noël</t>
         </is>
       </c>
       <c r="C201" s="2" t="n">
@@ -5459,12 +5459,12 @@
       </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
-          <t>Comment s’appelle la peur du vendredi 13 ?</t>
+          <t>Quel poème de 1823 a fixé l’image du traîneau tiré par des rennes ?</t>
         </is>
       </c>
       <c r="E201" s="3" t="inlineStr">
         <is>
-          <t>La paraskevidékatriaphobie</t>
+          <t>« A Visit from St. Nicholas » (« La Nuit avant Noël »)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Description courte sous le nom de chaque booster
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4e3JGtiCx8jxBb2JR7Gh3
</commit_message>
<xml_diff>
--- a/themes.xlsx
+++ b/themes.xlsx
@@ -6769,7 +6769,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ce qu’on sort au bar pour briller.</t>
+          <t>Monuments, histoire et grands événements</t>
         </is>
       </c>
     </row>
@@ -6786,7 +6786,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Meubles en kit, raclette et bulles.</t>
+          <t>Vie d’adulte : maison, bouffe, bagnole</t>
         </is>
       </c>
     </row>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Films, séries et idoles de la pop.</t>
+          <t>Films, séries, musique et pop culture</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pour ceux qui ont eu une Game Boy.</t>
+          <t>Pop culture des années 90</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Du savoir qui ne sert à rien, donc indispensable.</t>
+          <t>Anecdotes et savoirs improbables</t>
         </is>
       </c>
     </row>

</xml_diff>